<commit_message>
[IMP] puentes del planificador: paquete 1.8
Cuadrillas por día y asistencia (crew, attendance), control de consumo y
tablero sin montos (purchase, budget, mrp), repetición, re-trabajo y
porcentaje manual (subcontract, sale), catálogo de mobiliario, productos
por módulo, receta real, despacho e importador de la proyección
(furniture) y hoja de trabajo de la oficina técnica (spreadsheet).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016s9ZFwLqRQs1vnVc1jJkq3
</commit_message>
<xml_diff>
--- a/OL-PROJECTS/al_construction_planner_furniture/static/examples/eto_ejemplo.xlsx
+++ b/OL-PROJECTS/al_construction_planner_furniture/static/examples/eto_ejemplo.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A90"/>
+  <dimension ref="A1:A153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -732,7 +732,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Actividad de armado *: Código de una actividad que se mide por módulo.</t>
+          <t xml:space="preserve">  Actividad de armado: Código de una actividad que se mide por módulo; vacía: la del catálogo por el método de unión o el tipo de módulo.</t>
         </is>
       </c>
     </row>
@@ -744,281 +744,690 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr"/>
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Nombre: Función y ancho (MOD LAVADERO 900).</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>ACTIVIDADES: Actividades por ambiente de cada tipología.</t>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tipo de módulo: Estándar o Especial.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Método de unión: Tornillo, Tarugo, Mixto, Minifix o Sin unión.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVIDADES: Actividades por ambiente de cada tipología.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Tipología *: Código de la tipología.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  Actividad *: Código de la actividad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Cantidad por ambiente *: Unidades de driver de un ambiente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
-        <is>
-          <t>BOM: Lista de materiales de un ambiente de cada tipología.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Tipología *: Código de la tipología.</t>
+          <t xml:space="preserve">  Cantidad por ambiente *: Unidades de driver de un ambiente.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Código del producto *: Referencia interna del producto.</t>
-        </is>
-      </c>
+      <c r="A56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Producto: Nombre (para crear el producto si no existe).</t>
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>BOM: Lista de materiales de un ambiente de cada tipología.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cantidad *: Cantidad por ambiente.</t>
+          <t xml:space="preserve">  Tipología *: Código de la tipología.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unidad: Unidad de la cantidad; vacía: la del producto.</t>
+          <t xml:space="preserve">  Código del producto *: Referencia interna del producto.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Etapa de consumo: Producción, Armado, Instalación o Acabado y entrega. Sin etapa no se aprueba el plan.</t>
+          <t xml:space="preserve">  Producto: Nombre (para crear el producto si no existe).</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Costo unitario: Costo del maestro: informativo y costo del producto si se crea.</t>
+          <t xml:space="preserve">  Cantidad *: Cantidad por ambiente.</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr"/>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Unidad: Unidad de la cantidad; vacía: la del producto.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>ARBOL: Árbol de la obra: agrupador › piso › unidad › ambiente.</t>
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Etapa de consumo: Producción, Armado, Instalación o Acabado y entrega. Sin etapa no se aprueba el plan.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Agrupador: Torre o etapa encima del piso (p. ej. «Torre A»); varios niveles separados por « / » (p. ej. «Etapa 1 / Torre A»). Vacío si la obra no tiene agrupadores.</t>
+          <t xml:space="preserve">  Costo unitario: Costo del maestro: informativo y costo del producto si se crea.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Piso *: Nombre del piso.</t>
+          <t xml:space="preserve">  Módulo: Código del módulo: la línea va a la receta de ese módulo (v1.8); vacío: la tipología.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Departamento *: Nombre del departamento.</t>
+          <t xml:space="preserve">  Categoría: Categoría del producto (informativa).</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Ambiente *: Nombre del ambiente.</t>
-        </is>
-      </c>
+      <c r="A67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Tipología: Código de la tipología del ambiente.</t>
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>PIEZAS: Despiece de cada módulo (v1.8).</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Tipo de unidad: Departamento, Nivel de dúplex, Ducto, Estacionamiento, Área común, Depósito, Local o Piloto. Vacío: Departamento.</t>
+          <t xml:space="preserve">  Tipología *: Código de la tipología.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr"/>
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Módulo *: Código del módulo.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="3" t="inlineStr">
-        <is>
-          <t>VARIANTES: Variantes de una unidad o ambiente frente a su tipología.</t>
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Cantidad *: Piezas iguales.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Agrupador: Torre o etapa, como en ÁRBOL.</t>
+          <t xml:space="preserve">  Largo (mm): Largo de la pieza.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Piso *: Piso de la unidad.</t>
+          <t xml:space="preserve">  Ancho (mm): Ancho de la pieza.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Departamento *: Unidad.</t>
+          <t xml:space="preserve">  Tipo de pieza *: COSTADO, BASE, PUERTA, FRENTE, TAPA…</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Ambiente: Vacío: todos los ambientes de la unidad.</t>
+          <t xml:space="preserve">  Color: Color o descripción.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Tipo *: Color, Excluir o Metrado.</t>
+          <t xml:space="preserve">  Categoría: Categoría del tablero.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Código del producto *: Material de la tipología.</t>
+          <t xml:space="preserve">  Código del producto: Tablero de la pieza.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Reemplazar por: Solo para Color: código del material nuevo.</t>
+          <t xml:space="preserve">  Cantos: Cantos de la pieza.</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Cantidad por ambiente: Solo para Metrado.</t>
-        </is>
-      </c>
+      <c r="A79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Nota: Por qué (p. ej. «el cliente pidió Rovere»).</t>
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>PRODUCTOS NUEVOS: Productos que aún no están en el maestro (v1.8).</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="inlineStr"/>
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Código provisional *: El que usan BOM y PIEZAS hasta crear el producto.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" s="3" t="inlineStr">
-        <is>
-          <t>ETO: Módulos reales de cada ambiente (código y ancho), del despiece de ingeniería.</t>
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Nombre *: Nombre completo del producto.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Agrupador: Torre o etapa del piso, como en ÁRBOL.</t>
+          <t xml:space="preserve">  Unidad: Unidad del producto.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Piso *: Piso del ambiente.</t>
+          <t xml:space="preserve">  Categoría: Categoría (último nivel) del maestro.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Departamento *: Departamento del ambiente.</t>
+          <t xml:space="preserve">  Costo estimado: Costo del producto al crearlo.</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Ambiente *: Ambiente.</t>
-        </is>
-      </c>
+      <c r="A86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Código del módulo *: El mismo código de la plantilla de la tipología.</t>
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>TARIFAS: Tarifas de contrata pactadas para la obra (v1.8).</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Tipo: Bajo, Alto, Cajonera, Campana, Repisero u Otro.</t>
+          <t xml:space="preserve">  Actividad *: Código de la actividad.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Ancho (mm) *: Ancho real del módulo.</t>
+          <t xml:space="preserve">  Tarifa *: Tarifa de la obra.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Contratista: Vacío: cualquier contrata de la obra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Retención %: Retención de la liquidación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Vigente desde: Fecha de inicio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Vigente hasta: Fecha de fin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Familia: Cocina y baño o Closet y cajones (por defecto cocina).</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>OBRA: Datos y condiciones de la obra (v1.8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Dato *: Inicio, Fin, Cliente, Adelanto %, Fondo de garantía %…</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Valor *: Valor del dato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>CONTRATOS: Contratos de la obra con el cliente (v1.8, con Ventas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Contrato *: Nombre del contrato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Cliente: Cliente del contrato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Adelanto %: Adelanto del contrato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Fondo de garantía %: Fondo de garantía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Plantilla de hitos: Nombre de la plantilla (hoja HITOS).</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>HITOS: Hitos de cobro por unidad (v1.8, con Ventas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Plantilla *: Nombre de la plantilla de hitos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Hito *: Nombre del hito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  % *: Porcentaje del precio de la unidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Etapa: Etapa terminada que lo dispara.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>VENTA: Precio de venta por tipología (v1.8, con Ventas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Contrato *: Contrato de la hoja CONTRATOS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tipología *: Código de la tipología.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Precio por ambiente *: Precio de un ambiente de la tipología.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>MO PROPIA: Mano de obra propia: roles de cuadrilla (v1.8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Rol *: Operario, oficial, peón…</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Categoría: Categoría de construcción civil.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sub etapa: Sub etapa donde trabaja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Jornal: Costo de referencia por jornal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Rendimiento: Unidades por jornal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Actividad: Actividad (driver) que ejecuta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>ARBOL: Árbol de la obra: agrupador › piso › unidad › ambiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Agrupador: Torre o etapa encima del piso (p. ej. «Torre A»); varios niveles separados por « / » (p. ej. «Etapa 1 / Torre A»). Vacío si la obra no tiene agrupadores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Piso *: Nombre del piso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Departamento *: Nombre del departamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ambiente *: Nombre del ambiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tipología: Código de la tipología del ambiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tipo de unidad: Departamento, Nivel de dúplex, Ducto, Estacionamiento, Área común, Depósito, Local o Piloto. Vacío: Departamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>VARIANTES: Variantes de una unidad o ambiente frente a su tipología.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Agrupador: Torre o etapa, como en ÁRBOL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Piso *: Piso de la unidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Departamento *: Unidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ambiente: Vacío: todos los ambientes de la unidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tipo *: Color, Excluir o Metrado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Código del producto *: Material de la tipología.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Reemplazar por: Solo para Color: código del material nuevo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Cantidad por ambiente: Solo para Metrado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Nota: Por qué (p. ej. «el cliente pidió Rovere»).</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>ETO: Módulos reales de cada ambiente (código y ancho), del despiece de ingeniería.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Agrupador: Torre o etapa del piso, como en ÁRBOL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Piso *: Piso del ambiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Departamento *: Departamento del ambiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ambiente *: Ambiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Código del módulo *: El mismo código de la plantilla de la tipología.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tipo: Bajo, Alto, Cajonera, Campana, Repisero u Otro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ancho (mm) *: Ancho real del módulo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  Grupo ML: Mueble bajo, Mueble alto o Sin ML.</t>
         </is>

</xml_diff>